<commit_message>
Formato DescargaObservacionesInspección - Nueva columna
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/DescargaObservacionesInspección.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/DescargaObservacionesInspección.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Rediseño\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\Inspecciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF35F5DF-1A8D-4741-9282-83D48781E28B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F562CBFB-4323-45C6-8DE6-85EB8F5129D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{059AFEB3-0035-408C-B41B-FD5A473A479F}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Observaciones" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Observaciones!$A:$T</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Observaciones!$A:$U</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Nro</t>
   </si>
@@ -91,6 +91,9 @@
   </si>
   <si>
     <t>Acto / Condición subestándar Identificada</t>
+  </si>
+  <si>
+    <t>Descripción de Condición / Acto Subestándar</t>
   </si>
 </sst>
 </file>
@@ -180,7 +183,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -476,31 +479,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17F4CCAF-D617-4718-A62C-D29B21C2BA16}">
-  <dimension ref="B1:S2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:T2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="43.7109375" customWidth="1"/>
-    <col min="6" max="6" width="31.5703125" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="30.7109375" customWidth="1"/>
-    <col min="9" max="9" width="29.5703125" customWidth="1"/>
-    <col min="10" max="10" width="19" customWidth="1"/>
-    <col min="11" max="11" width="43.7109375" customWidth="1"/>
-    <col min="12" max="12" width="16.42578125" customWidth="1"/>
-    <col min="13" max="13" width="20.5703125" customWidth="1"/>
-    <col min="14" max="14" width="41.140625" customWidth="1"/>
-    <col min="15" max="15" width="19" customWidth="1"/>
-    <col min="16" max="16" width="18.7109375" customWidth="1"/>
-    <col min="17" max="18" width="22" customWidth="1"/>
-    <col min="20" max="20" width="1.5703125" customWidth="1"/>
+    <col min="5" max="6" width="43.7109375" customWidth="1"/>
+    <col min="7" max="7" width="31.5703125" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="30.7109375" customWidth="1"/>
+    <col min="10" max="10" width="29.5703125" customWidth="1"/>
+    <col min="11" max="11" width="19" customWidth="1"/>
+    <col min="12" max="12" width="43.7109375" customWidth="1"/>
+    <col min="13" max="13" width="16.42578125" customWidth="1"/>
+    <col min="14" max="14" width="20.5703125" customWidth="1"/>
+    <col min="15" max="15" width="41.140625" customWidth="1"/>
+    <col min="16" max="16" width="19" customWidth="1"/>
+    <col min="17" max="17" width="18.7109375" customWidth="1"/>
+    <col min="18" max="19" width="22" customWidth="1"/>
+    <col min="21" max="21" width="1.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:19" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:19" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:20" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:20" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -514,45 +517,48 @@
         <v>2</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="Q2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="R2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="R2" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Añadir Asesor y Participantes de inspección en descarga
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/DescargaObservacionesInspección.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/DescargaObservacionesInspección.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25028"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Rediseño\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\Inspecciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F562CBFB-4323-45C6-8DE6-85EB8F5129D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C3B3446-F595-4A47-86D6-6324D1E184D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{059AFEB3-0035-408C-B41B-FD5A473A479F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{059AFEB3-0035-408C-B41B-FD5A473A479F}"/>
   </bookViews>
   <sheets>
     <sheet name="Observaciones" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Observaciones!$A:$U</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Observaciones!$A:$W</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Nro</t>
   </si>
@@ -94,6 +94,12 @@
   </si>
   <si>
     <t>Descripción de Condición / Acto Subestándar</t>
+  </si>
+  <si>
+    <t>Participantes de la inspección</t>
+  </si>
+  <si>
+    <t>Asesor (MAP/SSO)</t>
   </si>
 </sst>
 </file>
@@ -479,7 +485,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17F4CCAF-D617-4718-A62C-D29B21C2BA16}">
-  <dimension ref="B1:T2"/>
+  <dimension ref="B1:V2"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
@@ -498,12 +504,12 @@
     <col min="15" max="15" width="41.140625" customWidth="1"/>
     <col min="16" max="16" width="19" customWidth="1"/>
     <col min="17" max="17" width="18.7109375" customWidth="1"/>
-    <col min="18" max="19" width="22" customWidth="1"/>
-    <col min="21" max="21" width="1.5703125" customWidth="1"/>
+    <col min="18" max="21" width="22" customWidth="1"/>
+    <col min="23" max="23" width="1.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:20" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:20" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:22" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -559,6 +565,12 @@
         <v>13</v>
       </c>
       <c r="T2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V2" s="1" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nuevo gráfico y nuevos filtros en reportes de inspecciones
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/DescargaObservacionesInspección.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/DescargaObservacionesInspección.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Rediseño\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\Inspecciones\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Gestiona Marcobre\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\Inspecciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C3B3446-F595-4A47-86D6-6324D1E184D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8470D6C6-4E2F-4151-9143-7DB50EE68E78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{059AFEB3-0035-408C-B41B-FD5A473A479F}"/>
+    <workbookView xWindow="4290" yWindow="4515" windowWidth="28800" windowHeight="15345" xr2:uid="{059AFEB3-0035-408C-B41B-FD5A473A479F}"/>
   </bookViews>
   <sheets>
     <sheet name="Observaciones" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Observaciones!$A:$W</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Observaciones!$A:$X</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Nro</t>
   </si>
@@ -100,6 +100,9 @@
   </si>
   <si>
     <t>Asesor (MAP/SSO)</t>
+  </si>
+  <si>
+    <t>Área Inspeccionada</t>
   </si>
 </sst>
 </file>
@@ -189,9 +192,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -229,7 +232,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -335,7 +338,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -477,7 +480,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -485,7 +488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17F4CCAF-D617-4718-A62C-D29B21C2BA16}">
-  <dimension ref="B1:V2"/>
+  <dimension ref="B1:W2"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
@@ -502,14 +505,14 @@
     <col min="13" max="13" width="16.42578125" customWidth="1"/>
     <col min="14" max="14" width="20.5703125" customWidth="1"/>
     <col min="15" max="15" width="41.140625" customWidth="1"/>
-    <col min="16" max="16" width="19" customWidth="1"/>
-    <col min="17" max="17" width="18.7109375" customWidth="1"/>
-    <col min="18" max="21" width="22" customWidth="1"/>
-    <col min="23" max="23" width="1.5703125" customWidth="1"/>
+    <col min="16" max="17" width="19" customWidth="1"/>
+    <col min="18" max="18" width="18.7109375" customWidth="1"/>
+    <col min="19" max="22" width="22" customWidth="1"/>
+    <col min="24" max="24" width="1.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:22" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:23" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:23" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -556,21 +559,24 @@
         <v>10</v>
       </c>
       <c r="Q2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="R2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="R2" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="U2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U2" s="1" t="s">
+      <c r="V2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="W2" s="1" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización de descarga de observaciones
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/DescargaObservacionesInspección.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/DescargaObservacionesInspección.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Gestiona Marcobre\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\Inspecciones\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\Inspecciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8470D6C6-4E2F-4151-9143-7DB50EE68E78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3AB787E-2E6D-4C77-8422-10E77B4CF370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="4515" windowWidth="28800" windowHeight="15345" xr2:uid="{059AFEB3-0035-408C-B41B-FD5A473A479F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{059AFEB3-0035-408C-B41B-FD5A473A479F}"/>
   </bookViews>
   <sheets>
     <sheet name="Observaciones" sheetId="1" r:id="rId1"/>
@@ -66,9 +66,6 @@
     <t>Estado</t>
   </si>
   <si>
-    <t>Responsable Inspección</t>
-  </si>
-  <si>
     <t>Fecha Inspección</t>
   </si>
   <si>
@@ -103,6 +100,9 @@
   </si>
   <si>
     <t>Área Inspeccionada</t>
+  </si>
+  <si>
+    <t>Líder de Inspección</t>
   </si>
 </sst>
 </file>
@@ -520,22 +520,22 @@
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>4</v>
@@ -553,31 +553,31 @@
         <v>8</v>
       </c>
       <c r="O2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="P2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="Q2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="R2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="Q2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="R2" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="U2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="W2" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cambio de nombre carpeta descargas, actualización descarga inspecciones y corrección de TextArea
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/DescargaObservacionesInspección.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/DescargaObservacionesInspección.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Gestiona Marcobre\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\Inspecciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8470D6C6-4E2F-4151-9143-7DB50EE68E78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D119A7C-2D81-49EA-9C78-9BA76F9CE351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="4515" windowWidth="28800" windowHeight="15345" xr2:uid="{059AFEB3-0035-408C-B41B-FD5A473A479F}"/>
+    <workbookView xWindow="0" yWindow="10410" windowWidth="38400" windowHeight="10470" xr2:uid="{059AFEB3-0035-408C-B41B-FD5A473A479F}"/>
   </bookViews>
   <sheets>
     <sheet name="Observaciones" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Observaciones!$A:$X</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Observaciones!$A:$Y</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Nro</t>
   </si>
@@ -66,9 +66,6 @@
     <t>Estado</t>
   </si>
   <si>
-    <t>Responsable Inspección</t>
-  </si>
-  <si>
     <t>Fecha Inspección</t>
   </si>
   <si>
@@ -103,6 +100,12 @@
   </si>
   <si>
     <t>Área Inspeccionada</t>
+  </si>
+  <si>
+    <t>Lider de la Inspección</t>
+  </si>
+  <si>
+    <t>Tipo de Inspección</t>
   </si>
 </sst>
 </file>
@@ -488,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17F4CCAF-D617-4718-A62C-D29B21C2BA16}">
-  <dimension ref="B1:W2"/>
+  <dimension ref="B1:X2"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
@@ -507,12 +510,13 @@
     <col min="15" max="15" width="41.140625" customWidth="1"/>
     <col min="16" max="17" width="19" customWidth="1"/>
     <col min="18" max="18" width="18.7109375" customWidth="1"/>
-    <col min="19" max="22" width="22" customWidth="1"/>
-    <col min="24" max="24" width="1.5703125" customWidth="1"/>
+    <col min="19" max="23" width="22" customWidth="1"/>
+    <col min="24" max="24" width="17.5703125" customWidth="1"/>
+    <col min="25" max="25" width="1.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:23" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:23" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:24" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -520,22 +524,22 @@
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>4</v>
@@ -553,31 +557,34 @@
         <v>8</v>
       </c>
       <c r="O2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="P2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="Q2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="R2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="Q2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="R2" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="U2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X2" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Descarga de FlashReport y Notificaciones agregadas
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/DescargaObservacionesInspección.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/DescargaObservacionesInspección.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Gestiona Marcobre\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\Inspecciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D119A7C-2D81-49EA-9C78-9BA76F9CE351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{198CA5D0-C762-4AB9-817B-C982EC928A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="10410" windowWidth="38400" windowHeight="10470" xr2:uid="{059AFEB3-0035-408C-B41B-FD5A473A479F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{059AFEB3-0035-408C-B41B-FD5A473A479F}"/>
   </bookViews>
   <sheets>
     <sheet name="Observaciones" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Observaciones!$A:$Y</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Observaciones!$A:$Z</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcOnSave="0" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Nro</t>
   </si>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t>Tipo de Inspección</t>
+  </si>
+  <si>
+    <t>Empresa Inspeccionada</t>
   </si>
 </sst>
 </file>
@@ -195,7 +198,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -491,32 +494,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17F4CCAF-D617-4718-A62C-D29B21C2BA16}">
-  <dimension ref="B1:X2"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:Y2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" customWidth="1"/>
+    <col min="1" max="1" width="1.7265625" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="43.7109375" customWidth="1"/>
-    <col min="7" max="7" width="31.5703125" customWidth="1"/>
+    <col min="3" max="3" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="43.7265625" customWidth="1"/>
+    <col min="7" max="7" width="31.54296875" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="30.7109375" customWidth="1"/>
-    <col min="10" max="10" width="29.5703125" customWidth="1"/>
+    <col min="9" max="9" width="30.7265625" customWidth="1"/>
+    <col min="10" max="10" width="29.54296875" customWidth="1"/>
     <col min="11" max="11" width="19" customWidth="1"/>
-    <col min="12" max="12" width="43.7109375" customWidth="1"/>
-    <col min="13" max="13" width="16.42578125" customWidth="1"/>
-    <col min="14" max="14" width="20.5703125" customWidth="1"/>
-    <col min="15" max="15" width="41.140625" customWidth="1"/>
+    <col min="12" max="12" width="43.7265625" customWidth="1"/>
+    <col min="13" max="13" width="16.453125" customWidth="1"/>
+    <col min="14" max="14" width="20.54296875" customWidth="1"/>
+    <col min="15" max="15" width="41.1796875" customWidth="1"/>
     <col min="16" max="17" width="19" customWidth="1"/>
-    <col min="18" max="18" width="18.7109375" customWidth="1"/>
-    <col min="19" max="23" width="22" customWidth="1"/>
-    <col min="24" max="24" width="17.5703125" customWidth="1"/>
-    <col min="25" max="25" width="1.5703125" customWidth="1"/>
+    <col min="18" max="18" width="18.7265625" customWidth="1"/>
+    <col min="19" max="24" width="22" customWidth="1"/>
+    <col min="25" max="25" width="17.54296875" customWidth="1"/>
+    <col min="26" max="26" width="1.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:24" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:25" ht="6" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:25" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -575,15 +578,18 @@
         <v>12</v>
       </c>
       <c r="U2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="V2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="W2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="X2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X2" s="1" t="s">
+      <c r="Y2" s="1" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>